<commit_message>
Increase number of datasets
</commit_message>
<xml_diff>
--- a/comparison_metrics/comparison_metrics_medium.xlsx
+++ b/comparison_metrics/comparison_metrics_medium.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:J338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11280,6 +11280,1338 @@
         <v>0.8590511458468578</v>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>CP.nex</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>6</v>
+      </c>
+      <c r="D302" t="n">
+        <v>29</v>
+      </c>
+      <c r="E302" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F302" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="G302" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H302" t="n">
+        <v>0.2758620689655172</v>
+      </c>
+      <c r="I302" t="n">
+        <v>0.6990740740740741</v>
+      </c>
+      <c r="J302" t="n">
+        <v>0.9630035054558818</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>IFL.nex</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>17</v>
+      </c>
+      <c r="D303" t="n">
+        <v>17</v>
+      </c>
+      <c r="E303" t="n">
+        <v>0.2941176470588235</v>
+      </c>
+      <c r="F303" t="n">
+        <v>0.2941176470588235</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0.3079584775086505</v>
+      </c>
+      <c r="H303" t="n">
+        <v>0.3217993079584775</v>
+      </c>
+      <c r="I303" t="n">
+        <v>0.9112946734123692</v>
+      </c>
+      <c r="J303" t="n">
+        <v>0.6799158268007248</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>COG3715.nex</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>100</v>
+      </c>
+      <c r="D304" t="n">
+        <v>40</v>
+      </c>
+      <c r="E304" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F304" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0.0859</v>
+      </c>
+      <c r="H304" t="n">
+        <v>0.235625</v>
+      </c>
+      <c r="I304" t="n">
+        <v>0.545058494546282</v>
+      </c>
+      <c r="J304" t="n">
+        <v>0.9736384834424484</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Wolbacchia.nex</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>387</v>
+      </c>
+      <c r="D305" t="n">
+        <v>387</v>
+      </c>
+      <c r="E305" t="n">
+        <v>0.3023255813953488</v>
+      </c>
+      <c r="F305" t="n">
+        <v>0.1834625322997416</v>
+      </c>
+      <c r="G305" t="n">
+        <v>0.0346266583872497</v>
+      </c>
+      <c r="H305" t="n">
+        <v>0.05274122148108087</v>
+      </c>
+      <c r="I305" t="n">
+        <v>0.8371749423807486</v>
+      </c>
+      <c r="J305" t="n">
+        <v>0.9972956133428755</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>CA.nex</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>41</v>
+      </c>
+      <c r="D306" t="n">
+        <v>30</v>
+      </c>
+      <c r="E306" t="n">
+        <v>0.3170731707317073</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0.2666666666666667</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0.1915526472337894</v>
+      </c>
+      <c r="H306" t="n">
+        <v>0.1988888888888889</v>
+      </c>
+      <c r="I306" t="n">
+        <v>0.7654208968701927</v>
+      </c>
+      <c r="J306" t="n">
+        <v>0.8011111111111112</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>CT.nex</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>19</v>
+      </c>
+      <c r="D307" t="n">
+        <v>19</v>
+      </c>
+      <c r="E307" t="n">
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0.2631578947368421</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0.3296398891966759</v>
+      </c>
+      <c r="H307" t="n">
+        <v>0.3379501385041551</v>
+      </c>
+      <c r="I307" t="n">
+        <v>0.9300368742366441</v>
+      </c>
+      <c r="J307" t="n">
+        <v>0.9401805700314609</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>datset_ficus.nex</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>204</v>
+      </c>
+      <c r="D308" t="n">
+        <v>153</v>
+      </c>
+      <c r="E308" t="n">
+        <v>0.3284313725490196</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0.2875816993464052</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0.06862745098039216</v>
+      </c>
+      <c r="H308" t="n">
+        <v>0.101200393011235</v>
+      </c>
+      <c r="I308" t="n">
+        <v>0.9950496250455846</v>
+      </c>
+      <c r="J308" t="n">
+        <v>0.9933760746818342</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>RM.nex</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>5</v>
+      </c>
+      <c r="D309" t="n">
+        <v>5</v>
+      </c>
+      <c r="E309" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="H309" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="I309" t="n">
+        <v>0.6879999999999999</v>
+      </c>
+      <c r="J309" t="n">
+        <v>0.6879999999999999</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>GL.nex</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>8</v>
+      </c>
+      <c r="D310" t="n">
+        <v>10</v>
+      </c>
+      <c r="E310" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0.46875</v>
+      </c>
+      <c r="H310" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I310" t="n">
+        <v>0.568878173828125</v>
+      </c>
+      <c r="J310" t="n">
+        <v>0.624</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>COG4964.nex</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>100</v>
+      </c>
+      <c r="D311" t="n">
+        <v>27</v>
+      </c>
+      <c r="E311" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0.2962962962962963</v>
+      </c>
+      <c r="G311" t="n">
+        <v>0.0859</v>
+      </c>
+      <c r="H311" t="n">
+        <v>0.2386831275720165</v>
+      </c>
+      <c r="I311" t="n">
+        <v>0.545058494546282</v>
+      </c>
+      <c r="J311" t="n">
+        <v>0.9458648122201924</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>COG4965.nex</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>100</v>
+      </c>
+      <c r="D312" t="n">
+        <v>30</v>
+      </c>
+      <c r="E312" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G312" t="n">
+        <v>0.0859</v>
+      </c>
+      <c r="H312" t="n">
+        <v>0.2522222222222222</v>
+      </c>
+      <c r="I312" t="n">
+        <v>0.545058494546282</v>
+      </c>
+      <c r="J312" t="n">
+        <v>0.6942091130378024</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>GM.nex</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>14</v>
+      </c>
+      <c r="D313" t="n">
+        <v>14</v>
+      </c>
+      <c r="E313" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="F313" t="n">
+        <v>0.2142857142857143</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0.3418367346938775</v>
+      </c>
+      <c r="H313" t="n">
+        <v>0.3622448979591837</v>
+      </c>
+      <c r="I313" t="n">
+        <v>0.8838543304660472</v>
+      </c>
+      <c r="J313" t="n">
+        <v>0.8941143347250842</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>COG2085.nex</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>100</v>
+      </c>
+      <c r="D314" t="n">
+        <v>44</v>
+      </c>
+      <c r="E314" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="G314" t="n">
+        <v>0.0859</v>
+      </c>
+      <c r="H314" t="n">
+        <v>0.2004132231404959</v>
+      </c>
+      <c r="I314" t="n">
+        <v>0.545058494546282</v>
+      </c>
+      <c r="J314" t="n">
+        <v>0.8371966390980969</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>PP.nex</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>36</v>
+      </c>
+      <c r="D315" t="n">
+        <v>41</v>
+      </c>
+      <c r="E315" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F315" t="n">
+        <v>0.2682926829268293</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0.1604938271604938</v>
+      </c>
+      <c r="H315" t="n">
+        <v>0.1516954193932183</v>
+      </c>
+      <c r="I315" t="n">
+        <v>0.5619708469684025</v>
+      </c>
+      <c r="J315" t="n">
+        <v>0.5652762017191585</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>PML.nex</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>18</v>
+      </c>
+      <c r="D316" t="n">
+        <v>18</v>
+      </c>
+      <c r="E316" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F316" t="n">
+        <v>0.3888888888888889</v>
+      </c>
+      <c r="G316" t="n">
+        <v>0.3055555555555556</v>
+      </c>
+      <c r="H316" t="n">
+        <v>0.2839506172839506</v>
+      </c>
+      <c r="I316" t="n">
+        <v>0.8149112523649014</v>
+      </c>
+      <c r="J316" t="n">
+        <v>0.7792093513202782</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>EC.nex</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>7</v>
+      </c>
+      <c r="D317" t="n">
+        <v>10</v>
+      </c>
+      <c r="E317" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="F317" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G317" t="n">
+        <v>0.4693877551020408</v>
+      </c>
+      <c r="H317" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I317" t="n">
+        <v>0.7551020408163265</v>
+      </c>
+      <c r="J317" t="n">
+        <v>0.876502</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>RH.nex</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>34</v>
+      </c>
+      <c r="D318" t="n">
+        <v>42</v>
+      </c>
+      <c r="E318" t="n">
+        <v>0.3823529411764706</v>
+      </c>
+      <c r="F318" t="n">
+        <v>0.3095238095238095</v>
+      </c>
+      <c r="G318" t="n">
+        <v>0.1842560553633218</v>
+      </c>
+      <c r="H318" t="n">
+        <v>0.1729024943310657</v>
+      </c>
+      <c r="I318" t="n">
+        <v>0.6647730473277632</v>
+      </c>
+      <c r="J318" t="n">
+        <v>0.9622821387294426</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>SHA.nex</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>14</v>
+      </c>
+      <c r="D319" t="n">
+        <v>16</v>
+      </c>
+      <c r="E319" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="F319" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="G319" t="n">
+        <v>0.2806122448979592</v>
+      </c>
+      <c r="H319" t="n">
+        <v>0.27734375</v>
+      </c>
+      <c r="I319" t="n">
+        <v>0.02116305705955852</v>
+      </c>
+      <c r="J319" t="n">
+        <v>0.6414041519165039</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>FA.nex</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>7</v>
+      </c>
+      <c r="D320" t="n">
+        <v>8</v>
+      </c>
+      <c r="E320" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="F320" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="G320" t="n">
+        <v>0.4693877551020408</v>
+      </c>
+      <c r="H320" t="n">
+        <v>0.40625</v>
+      </c>
+      <c r="I320" t="n">
+        <v>0.4960433152852978</v>
+      </c>
+      <c r="J320" t="n">
+        <v>0.50390625</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>tahiti_araneae_coleoptera_odonata.nex</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>12</v>
+      </c>
+      <c r="D321" t="n">
+        <v>12</v>
+      </c>
+      <c r="E321" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F321" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="G321" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H321" t="n">
+        <v>0.4930555555555556</v>
+      </c>
+      <c r="I321" t="n">
+        <v>0.3641050990226337</v>
+      </c>
+      <c r="J321" t="n">
+        <v>0.900725611546342</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>SC.nex</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>11</v>
+      </c>
+      <c r="D322" t="n">
+        <v>14</v>
+      </c>
+      <c r="E322" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="F322" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="G322" t="n">
+        <v>0.4049586776859504</v>
+      </c>
+      <c r="H322" t="n">
+        <v>0.3571428571428572</v>
+      </c>
+      <c r="I322" t="n">
+        <v>0.8544628155620946</v>
+      </c>
+      <c r="J322" t="n">
+        <v>0.8940604137397805</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>RP.nex</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>13</v>
+      </c>
+      <c r="D323" t="n">
+        <v>13</v>
+      </c>
+      <c r="E323" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="F323" t="n">
+        <v>0.2307692307692308</v>
+      </c>
+      <c r="G323" t="n">
+        <v>0.3668639053254438</v>
+      </c>
+      <c r="H323" t="n">
+        <v>0.3550295857988165</v>
+      </c>
+      <c r="I323" t="n">
+        <v>0.5932650487978863</v>
+      </c>
+      <c r="J323" t="n">
+        <v>0.2873877959538072</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>SSA.nex</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>10</v>
+      </c>
+      <c r="D324" t="n">
+        <v>10</v>
+      </c>
+      <c r="E324" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F324" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G324" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="H324" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I324" t="n">
+        <v>0.4429999999999999</v>
+      </c>
+      <c r="J324" t="n">
+        <v>0.4643</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>SFC.nex</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>15</v>
+      </c>
+      <c r="D325" t="n">
+        <v>16</v>
+      </c>
+      <c r="E325" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F325" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G325" t="n">
+        <v>0.3288888888888889</v>
+      </c>
+      <c r="H325" t="n">
+        <v>0.3828125</v>
+      </c>
+      <c r="I325" t="n">
+        <v>0.8951533388203018</v>
+      </c>
+      <c r="J325" t="n">
+        <v>0.9282611685339361</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>FD.nex</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>20</v>
+      </c>
+      <c r="D326" t="n">
+        <v>51</v>
+      </c>
+      <c r="E326" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F326" t="n">
+        <v>0.3725490196078431</v>
+      </c>
+      <c r="G326" t="n">
+        <v>0.3575</v>
+      </c>
+      <c r="H326" t="n">
+        <v>0.170319108035371</v>
+      </c>
+      <c r="I326" t="n">
+        <v>0.9342035992598634</v>
+      </c>
+      <c r="J326" t="n">
+        <v>0.7000143027767055</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>SFC_c.nex</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
+        <v>15</v>
+      </c>
+      <c r="D327" t="n">
+        <v>16</v>
+      </c>
+      <c r="E327" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F327" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G327" t="n">
+        <v>0.3288888888888889</v>
+      </c>
+      <c r="H327" t="n">
+        <v>0.3828125</v>
+      </c>
+      <c r="I327" t="n">
+        <v>0.8951533388203018</v>
+      </c>
+      <c r="J327" t="n">
+        <v>0.9282611685339361</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>PMP.nex</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>18</v>
+      </c>
+      <c r="D328" t="n">
+        <v>18</v>
+      </c>
+      <c r="E328" t="n">
+        <v>0.2777777777777778</v>
+      </c>
+      <c r="F328" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0.3179012345679013</v>
+      </c>
+      <c r="H328" t="n">
+        <v>0.3271604938271605</v>
+      </c>
+      <c r="I328" t="n">
+        <v>0.8149134020096153</v>
+      </c>
+      <c r="J328" t="n">
+        <v>0.8159236874801281</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>FE.nex</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>5</v>
+      </c>
+      <c r="D329" t="n">
+        <v>5</v>
+      </c>
+      <c r="E329" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F329" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="H329" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="I329" t="n">
+        <v>0.6879999999999999</v>
+      </c>
+      <c r="J329" t="n">
+        <v>0.6879999999999999</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>CP_1.nex</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>6</v>
+      </c>
+      <c r="D330" t="n">
+        <v>29</v>
+      </c>
+      <c r="E330" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F330" t="n">
+        <v>0.3448275862068966</v>
+      </c>
+      <c r="G330" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H330" t="n">
+        <v>0.2758620689655172</v>
+      </c>
+      <c r="I330" t="n">
+        <v>0.6990740740740741</v>
+      </c>
+      <c r="J330" t="n">
+        <v>0.9630035054558818</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>AP.nex</t>
+        </is>
+      </c>
+      <c r="C331" t="n">
+        <v>10</v>
+      </c>
+      <c r="D331" t="n">
+        <v>7</v>
+      </c>
+      <c r="E331" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F331" t="n">
+        <v>0.1428571428571428</v>
+      </c>
+      <c r="G331" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H331" t="n">
+        <v>0.5510204081632653</v>
+      </c>
+      <c r="I331" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="J331" t="n">
+        <v>0.805557208306063</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>SBL.nex</t>
+        </is>
+      </c>
+      <c r="C332" t="n">
+        <v>15</v>
+      </c>
+      <c r="D332" t="n">
+        <v>8</v>
+      </c>
+      <c r="E332" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="F332" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G332" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H332" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I332" t="n">
+        <v>0.8957656844993142</v>
+      </c>
+      <c r="J332" t="n">
+        <v>0.832550048828125</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>TD.nex</t>
+        </is>
+      </c>
+      <c r="C333" t="n">
+        <v>26</v>
+      </c>
+      <c r="D333" t="n">
+        <v>22</v>
+      </c>
+      <c r="E333" t="n">
+        <v>0.3076923076923077</v>
+      </c>
+      <c r="F333" t="n">
+        <v>0.4090909090909091</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0.2736686390532544</v>
+      </c>
+      <c r="H333" t="n">
+        <v>0.2582644628099173</v>
+      </c>
+      <c r="I333" t="n">
+        <v>0.958372087786369</v>
+      </c>
+      <c r="J333" t="n">
+        <v>0.84770180260516</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>MF.nex</t>
+        </is>
+      </c>
+      <c r="C334" t="n">
+        <v>11</v>
+      </c>
+      <c r="D334" t="n">
+        <v>9</v>
+      </c>
+      <c r="E334" t="n">
+        <v>0.3636363636363636</v>
+      </c>
+      <c r="F334" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0.3884297520661157</v>
+      </c>
+      <c r="H334" t="n">
+        <v>0.3580246913580247</v>
+      </c>
+      <c r="I334" t="n">
+        <v>0.516289870910457</v>
+      </c>
+      <c r="J334" t="n">
+        <v>0.1248285322359396</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>AS.nex</t>
+        </is>
+      </c>
+      <c r="C335" t="n">
+        <v>19</v>
+      </c>
+      <c r="D335" t="n">
+        <v>16</v>
+      </c>
+      <c r="E335" t="n">
+        <v>0.4210526315789473</v>
+      </c>
+      <c r="F335" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0.2437673130193906</v>
+      </c>
+      <c r="H335" t="n">
+        <v>0.30078125</v>
+      </c>
+      <c r="I335" t="n">
+        <v>0.3830392293004355</v>
+      </c>
+      <c r="J335" t="n">
+        <v>0.6497527398169041</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>MP.nex</t>
+        </is>
+      </c>
+      <c r="C336" t="n">
+        <v>14</v>
+      </c>
+      <c r="D336" t="n">
+        <v>8</v>
+      </c>
+      <c r="E336" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="F336" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0.3469387755102041</v>
+      </c>
+      <c r="H336" t="n">
+        <v>0.484375</v>
+      </c>
+      <c r="I336" t="n">
+        <v>0.8846333957364704</v>
+      </c>
+      <c r="J336" t="n">
+        <v>0.83203125</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>AW.nex</t>
+        </is>
+      </c>
+      <c r="C337" t="n">
+        <v>12</v>
+      </c>
+      <c r="D337" t="n">
+        <v>12</v>
+      </c>
+      <c r="E337" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F337" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="G337" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H337" t="n">
+        <v>0.4930555555555556</v>
+      </c>
+      <c r="I337" t="n">
+        <v>0.3641050990226337</v>
+      </c>
+      <c r="J337" t="n">
+        <v>0.900725611546342</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Real_Data</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>TC.nex</t>
+        </is>
+      </c>
+      <c r="C338" t="n">
+        <v>8</v>
+      </c>
+      <c r="D338" t="n">
+        <v>9</v>
+      </c>
+      <c r="E338" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F338" t="n">
+        <v>0.2222222222222222</v>
+      </c>
+      <c r="G338" t="n">
+        <v>0.40625</v>
+      </c>
+      <c r="H338" t="n">
+        <v>0.4691358024691358</v>
+      </c>
+      <c r="I338" t="n">
+        <v>0.53125</v>
+      </c>
+      <c r="J338" t="n">
+        <v>0.8536977764229707</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>